<commit_message>
Append new quiz score
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,31 @@
         </is>
       </c>
       <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>fdggd</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>rgdtf</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>fdg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>sfr</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>